<commit_message>
paper run 2026-09-19 11:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-19.xlsx
+++ b/reports/2026-09-19.xlsx
@@ -632,13 +632,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>70.90000000000001</v>
+        <v>9.92</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -696,13 +696,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>-22</v>
+        <v>-82.98</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -722,13 +722,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>-60.98</v>
+        <v>-121.96</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C24" t="n">
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>9.92</v>
+        <v>-51.06</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>

</xml_diff>